<commit_message>
feat(qlcl): bo sung theo doi tan suat thi nghiem cot thep boc tach chi tiet tung thanh cho Cau Km19+529.080
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/260920_TDTC_CaXe_CaMay_DauDiezel_Cau_Km19+529.080.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/260920_TDTC_CaXe_CaMay_DauDiezel_Cau_Km19+529.080.xlsx
@@ -755,7 +755,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:GC70"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -38435,7 +38435,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -39122,7 +39122,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -39741,7 +39741,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -40196,7 +40196,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>

</xml_diff>